<commit_message>
v2.1.0: baris Edit KBLI = 0 diberi catatan #0 tanpa perubahan isian
</commit_message>
<xml_diff>
--- a/template-pengecekan-kbli.xlsx
+++ b/template-pengecekan-kbli.xlsx
@@ -8569,7 +8569,7 @@
   </sheetData>
   <autoFilter ref="A1:O2"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Edit KBLI" error="Isi 1 (dikoreksi) atau 0 / kosong (dilewati)." type="list">
+    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Edit KBLI" error="Isi 1 (dikoreksi), 0 (hanya catatan #0), atau kosong (dilewati)." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9005,7 +9005,7 @@
       <c r="N6" s="4" t="inlineStr"/>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>contoh: Edit KBLI bukan 1 → dilewati</t>
+          <t>contoh: Edit KBLI = 0 → tidak diubah, hanya catatan #0</t>
         </is>
       </c>
     </row>
@@ -16988,7 +16988,7 @@
   </sheetData>
   <autoFilter ref="A1:O6"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Edit KBLI" error="Isi 1 (dikoreksi) atau 0 / kosong (dilewati)." type="list">
+    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Edit KBLI" error="Isi 1 (dikoreksi), 0 (hanya catatan #0), atau kosong (dilewati)." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17224,7 +17224,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Isi 1 untuk baris yang mau dikoreksi. Baris selain 1 (termasuk kosong) dilewati.</t>
+          <t>1 = dikoreksi (KBLI/produk/kegiatan utama diganti). 0 = KBLI sudah benar: tidak ada yang diubah, kartu hanya diberi catatan #0 lalu Kirim &amp; Approve. Kosong = dilewati.</t>
         </is>
       </c>
     </row>

</xml_diff>